<commit_message>
creacion carpetas data y output
</commit_message>
<xml_diff>
--- a/output/estado_cuenta.xlsx
+++ b/output/estado_cuenta.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,706 +436,256 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>30/05</t>
+          <t>06/02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8119543 DIFERIDO INTERNACIONAL ONLINE (3/6)</t>
+          <t>28 CASH ADVANCE PREFERENTE 2 (7/60)</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>671.7</v>
+        <v>300.31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>30/05</t>
+          <t>22/07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8119546 DIFERIDO INTERNACIONAL ONLINE (3/6)</t>
+          <t>6797970 PLAN DEUDA ASEGURADA PLUS</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>327.12</v>
+        <v>8.66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>17/07</t>
+          <t>16/08</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8169587 DIFERIDO INTERNACIONAL ONLINE (2/6)</t>
+          <t>3276298 DN DTV*DIRECTVGO</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>122.28</v>
+        <v>19.99</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>28/11</t>
+          <t>16/08</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>994746 PTP - UNIVERSIDAD INTERNACIO (9/24)</t>
+          <t>3276298 RET IVA SERV DIGITAL 100%</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>110.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20/07</t>
+          <t>23/07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>9393961 EL CORTE INGLES M</t>
+          <t>2646070 AE Jack Jones</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>101.93</v>
+        <v>82.34999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20/07</t>
+          <t>18/07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9393961 CARGO CONSUMO EN EL EXTERIOR</t>
+          <t>2543750 63 Dlocal*UBER RIDES</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.7</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>20/07</t>
+          <t>18/07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9393962 GRAN VIA MADRID M</t>
+          <t>2543750 RET IVA SERV DIGITAL 100%</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>535.14</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20/07</t>
+          <t>16/08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9393962 CARGO CONSUMO EN EL EXTERIOR</t>
+          <t>3311592 63 Dlocal*UBER RIDES</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.7</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>21/07</t>
+          <t>16/08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9561089 FARMACIA BERNABE DEL AMOM</t>
+          <t>3311592 RET IVA SERV DIGITAL 100%</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>16.4</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>16/07</t>
+          <t>22/07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9024935 UBER RIDES S</t>
+          <t>2662872 018 MUeLLER KARLSRUHE 2-9 E</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2.33</v>
+        <v>82.70999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>16/07</t>
+          <t>18/08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9024935 RET IVA SERV DIGITAL 100%</t>
+          <t>IMPUESTO SALIDA DIVISAS</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.35</v>
+        <v>9.710000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>16/07</t>
+          <t>03/08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9024936 UBER RIDES S</t>
+          <t>15478 SU PAGO "MUCHAS GRACIAS"</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3.03</v>
+        <v>374.74</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>16/07</t>
+          <t>16/08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9024936 RET IVA SERV DIGITAL 100%</t>
+          <t>DN DTV*DIRECTVGO</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>17/07</t>
+          <t>23/07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9024937 UBER RIDES S</t>
+          <t>AE Jack Jones EUR</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4.07</v>
+        <v>69.98</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>17/07</t>
+          <t>18/07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>9024937 RET IVA SERV DIGITAL 100%</t>
+          <t>63 Dlocal*UBER RIDES</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>29/07</t>
+          <t>16/08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>593765 CRUNCHYROLL.COM C</t>
+          <t>63 Dlocal*UBER RIDES</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3.99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>29/07</t>
+          <t>22/07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>593765 RET IVA SERV DIGITAL 100%</t>
+          <t>018 MUeLLER KARLSRUHE 2-9 E EUR</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>20/07</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>9393960 PRIMOR PRECIADOS M</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>75.44</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>18/07</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>9103288 TPV ESIMFLAG EUR M</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>47.19</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>9561088 Chocolaterias 1902 II M</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>25.95</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>9561092 BARCA STORE MADRID E</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>165.1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>9561092 CARGO CONSUMO EN EL EXTERIOR</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>1.7</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>04/08</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>1336999 Zapping Ecuador S</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>9561091 MP**MARKET ALUCHE M</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>7.06</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>22/07</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>9658376 Urban Coffee F</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>27.63</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>9561090 TREBOL V</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>25.93</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>22/07</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>9658375 Miami Kiosk Karlsruhe K</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>15.29</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>18/08</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>3182709 Spotify P45CC4426F S</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>6.99</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>18/08</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>3182709 RET IVA SERV DIGITAL 100%</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>19/08</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>IMPUESTO SALIDA DIVISAS</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>53.09</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>03/08</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>10361 SU PAGO "MUCHAS GRACIAS"</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>1500.92</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>20/07</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>EL CORTE INGLES M EUR</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>86.40000000000001</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>20/07</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>GRAN VIA MADRID M EUR</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>453.6</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>FARMACIA BERNABE DEL AMOM EUR</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>13.9</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>16/07</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>UBER RIDES S</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>16/07</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>UBER RIDES S</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>17/07</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>UBER RIDES S</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>29/07</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>CRUNCHYROLL.COM C</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>20/07</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>PRIMOR PRECIADOS M EUR</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>63.94</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>18/07</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>TPV ESIMFLAG EUR M EUR</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Chocolaterias 1902 II M EUR</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>BARCA STORE MADRID E EUR</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>139.98</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>MP**MARKET ALUCHE M EUR</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>5.98</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>22/07</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Urban Coffee F</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>21/07</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>TREBOL V EUR</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>21.98</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>22/07</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Miami Kiosk Karlsruhe K EUR</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>12.98</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>18/08</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Spotify P45CC4426F S</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>0</v>
+        <v>70.29000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>